<commit_message>
1.5 | 1.6: Create and maintain product categories | populate db with products and associated categories
</commit_message>
<xml_diff>
--- a/Full Stack - Ecommerce Project Marking Sheet.xlsx
+++ b/Full Stack - Ecommerce Project Marking Sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6ea0a80ab323a6d7/Documents/TERM 3/WEBD-3011 Agile Full Stack Web Development/E-commerce Project/electrostore_app/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="5" documentId="11_48A0D02C31ED299F75CB867A24A221DF50C83E58" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7A310AAA-3046-49F4-9374-F0CE5EDA3520}"/>
+  <xr:revisionPtr revIDLastSave="7" documentId="11_48A0D02C31ED299F75CB867A24A221DF50C83E58" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{41FD56B6-851D-492C-8F95-3A108DAD2667}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1260,6 +1260,10 @@
 </styleSheet>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
@@ -1476,7 +1480,7 @@
     <row r="1" spans="1:29" ht="23.4" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="str">
         <f>"Unverified Marks: " &amp; I170 &amp; "  /  Verified: " &amp; J170 &amp; "  /  Verified with Deductions: " &amp; K170 &amp; "  /  Verified with Deductions &amp; Milestones: " &amp; L170</f>
-        <v>Unverified Marks: 4  /  Verified: 0  /  Verified with Deductions: -30  /  Verified with Deductions &amp; Milestones: -30</v>
+        <v>Unverified Marks: 8  /  Verified: 0  /  Verified with Deductions: -30  /  Verified with Deductions &amp; Milestones: -30</v>
       </c>
       <c r="C1" s="2"/>
       <c r="D1" s="3"/>
@@ -1650,7 +1654,7 @@
       </c>
       <c r="E5" s="10"/>
       <c r="F5" s="21" t="s">
-        <v>12</v>
+        <v>214</v>
       </c>
       <c r="G5" s="22">
         <v>2</v>
@@ -1660,7 +1664,7 @@
       </c>
       <c r="I5" s="24">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J5" s="24">
         <f t="shared" si="1"/>
@@ -1971,7 +1975,7 @@
       </c>
       <c r="E13" s="10"/>
       <c r="F13" s="21" t="s">
-        <v>12</v>
+        <v>214</v>
       </c>
       <c r="G13" s="22">
         <v>2</v>
@@ -1979,7 +1983,7 @@
       <c r="H13" s="10"/>
       <c r="I13" s="12">
         <f>IF(OR(F13 = "maybe", F13 = "yes"),G13, 0)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J13" s="12">
         <f>IF(F13 = "yes",G13, 0)</f>
@@ -7999,7 +8003,7 @@
       <c r="H170" s="10"/>
       <c r="I170" s="38">
         <f t="shared" ref="I170:K170" si="24">SUM(I4:I162)</f>
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="J170" s="12">
         <f t="shared" si="24"/>

</xml_diff>

<commit_message>
1.8 Extract seed data for products and categories from an existing  API.
</commit_message>
<xml_diff>
--- a/Full Stack - Ecommerce Project Marking Sheet.xlsx
+++ b/Full Stack - Ecommerce Project Marking Sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6ea0a80ab323a6d7/Documents/TERM 3/WEBD-3011 Agile Full Stack Web Development/E-commerce Project/electrostore_app/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="7" documentId="11_48A0D02C31ED299F75CB867A24A221DF50C83E58" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{41FD56B6-851D-492C-8F95-3A108DAD2667}"/>
+  <xr:revisionPtr revIDLastSave="9" documentId="11_48A0D02C31ED299F75CB867A24A221DF50C83E58" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{17DDB62E-B6DF-4517-A459-499DED97E266}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1480,7 +1480,7 @@
     <row r="1" spans="1:29" ht="23.4" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="str">
         <f>"Unverified Marks: " &amp; I170 &amp; "  /  Verified: " &amp; J170 &amp; "  /  Verified with Deductions: " &amp; K170 &amp; "  /  Verified with Deductions &amp; Milestones: " &amp; L170</f>
-        <v>Unverified Marks: 8  /  Verified: 0  /  Verified with Deductions: -30  /  Verified with Deductions &amp; Milestones: -30</v>
+        <v>Unverified Marks: 12  /  Verified: 0  /  Verified with Deductions: -30  /  Verified with Deductions &amp; Milestones: -30</v>
       </c>
       <c r="C1" s="2"/>
       <c r="D1" s="3"/>
@@ -2056,7 +2056,7 @@
       </c>
       <c r="E15" s="10"/>
       <c r="F15" s="21" t="s">
-        <v>12</v>
+        <v>214</v>
       </c>
       <c r="G15" s="22">
         <v>2</v>
@@ -2064,7 +2064,7 @@
       <c r="H15" s="23"/>
       <c r="I15" s="12">
         <f>IF(OR(F15 = "maybe", F15 = "yes"),G15, 0)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J15" s="12">
         <f>IF(F15 = "yes",G15, 0)</f>
@@ -2139,7 +2139,7 @@
       </c>
       <c r="E17" s="10"/>
       <c r="F17" s="21" t="s">
-        <v>12</v>
+        <v>214</v>
       </c>
       <c r="G17" s="22">
         <v>2</v>
@@ -2147,7 +2147,7 @@
       <c r="H17" s="23"/>
       <c r="I17" s="12">
         <f t="shared" ref="I17:I18" si="6">IF(OR(F17 = "maybe", F17 = "yes"),G17, 0)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J17" s="12">
         <f t="shared" ref="J17:J18" si="7">IF(F17 = "yes",G17, 0)</f>
@@ -8003,7 +8003,7 @@
       <c r="H170" s="10"/>
       <c r="I170" s="38">
         <f t="shared" ref="I170:K170" si="24">SUM(I4:I162)</f>
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="J170" s="12">
         <f t="shared" si="24"/>

</xml_diff>

<commit_message>
Add Category filter to Product admin page
</commit_message>
<xml_diff>
--- a/Full Stack - Ecommerce Project Marking Sheet.xlsx
+++ b/Full Stack - Ecommerce Project Marking Sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6ea0a80ab323a6d7/Documents/TERM 3/WEBD-3011 Agile Full Stack Web Development/E-commerce Project/electrostore_app/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="9" documentId="11_48A0D02C31ED299F75CB867A24A221DF50C83E58" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{17DDB62E-B6DF-4517-A459-499DED97E266}"/>
+  <xr:revisionPtr revIDLastSave="10" documentId="11_48A0D02C31ED299F75CB867A24A221DF50C83E58" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2C9ECDC7-17BA-4FC3-813E-7FB6EE38C0AD}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1480,7 +1480,7 @@
     <row r="1" spans="1:29" ht="23.4" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="str">
         <f>"Unverified Marks: " &amp; I170 &amp; "  /  Verified: " &amp; J170 &amp; "  /  Verified with Deductions: " &amp; K170 &amp; "  /  Verified with Deductions &amp; Milestones: " &amp; L170</f>
-        <v>Unverified Marks: 12  /  Verified: 0  /  Verified with Deductions: -30  /  Verified with Deductions &amp; Milestones: -30</v>
+        <v>Unverified Marks: 14  /  Verified: 0  /  Verified with Deductions: -30  /  Verified with Deductions &amp; Milestones: -30</v>
       </c>
       <c r="C1" s="2"/>
       <c r="D1" s="3"/>
@@ -2187,7 +2187,7 @@
       </c>
       <c r="E18" s="10"/>
       <c r="F18" s="21" t="s">
-        <v>12</v>
+        <v>214</v>
       </c>
       <c r="G18" s="22">
         <v>2</v>
@@ -2195,7 +2195,7 @@
       <c r="H18" s="23"/>
       <c r="I18" s="12">
         <f t="shared" si="6"/>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J18" s="12">
         <f t="shared" si="7"/>
@@ -8003,7 +8003,7 @@
       <c r="H170" s="10"/>
       <c r="I170" s="38">
         <f t="shared" ref="I170:K170" si="24">SUM(I4:I162)</f>
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="J170" s="12">
         <f t="shared" si="24"/>

</xml_diff>

<commit_message>
2.3: View the details of any of the available products on their own product page.
</commit_message>
<xml_diff>
--- a/Full Stack - Ecommerce Project Marking Sheet.xlsx
+++ b/Full Stack - Ecommerce Project Marking Sheet.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6ea0a80ab323a6d7/Documents/TERM 3/WEBD-3011 Agile Full Stack Web Development/E-commerce Project/electrostore_app/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\rndev\electrostore_app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="10" documentId="11_48A0D02C31ED299F75CB867A24A221DF50C83E58" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2C9ECDC7-17BA-4FC3-813E-7FB6EE38C0AD}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1421F2D7-81B6-4257-952A-C636E1A1C462}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1260,10 +1260,6 @@
 </styleSheet>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
@@ -1480,7 +1476,7 @@
     <row r="1" spans="1:29" ht="23.4" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="str">
         <f>"Unverified Marks: " &amp; I170 &amp; "  /  Verified: " &amp; J170 &amp; "  /  Verified with Deductions: " &amp; K170 &amp; "  /  Verified with Deductions &amp; Milestones: " &amp; L170</f>
-        <v>Unverified Marks: 14  /  Verified: 0  /  Verified with Deductions: -30  /  Verified with Deductions &amp; Milestones: -30</v>
+        <v>Unverified Marks: 16  /  Verified: 0  /  Verified with Deductions: -30  /  Verified with Deductions &amp; Milestones: -30</v>
       </c>
       <c r="C1" s="2"/>
       <c r="D1" s="3"/>
@@ -2336,7 +2332,7 @@
       </c>
       <c r="E22" s="10"/>
       <c r="F22" s="21" t="s">
-        <v>12</v>
+        <v>214</v>
       </c>
       <c r="G22" s="22">
         <v>2</v>
@@ -2346,7 +2342,7 @@
       </c>
       <c r="I22" s="12">
         <f t="shared" ref="I22:I23" si="9">IF(OR(F22 = "maybe", F22 = "yes"),G22, 0)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J22" s="12">
         <f t="shared" ref="J22:J23" si="10">IF(F22 = "yes",G22, 0)</f>
@@ -8003,7 +7999,7 @@
       <c r="H170" s="10"/>
       <c r="I170" s="38">
         <f t="shared" ref="I170:K170" si="24">SUM(I4:I162)</f>
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="J170" s="12">
         <f t="shared" si="24"/>

</xml_diff>

<commit_message>
2.5: Products listing are paginated.
</commit_message>
<xml_diff>
--- a/Full Stack - Ecommerce Project Marking Sheet.xlsx
+++ b/Full Stack - Ecommerce Project Marking Sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\rndev\electrostore_app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1421F2D7-81B6-4257-952A-C636E1A1C462}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22B1ACEC-2571-45E2-BA3E-ED6C6C24A9AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1476,7 +1476,7 @@
     <row r="1" spans="1:29" ht="23.4" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="str">
         <f>"Unverified Marks: " &amp; I170 &amp; "  /  Verified: " &amp; J170 &amp; "  /  Verified with Deductions: " &amp; K170 &amp; "  /  Verified with Deductions &amp; Milestones: " &amp; L170</f>
-        <v>Unverified Marks: 16  /  Verified: 0  /  Verified with Deductions: -30  /  Verified with Deductions &amp; Milestones: -30</v>
+        <v>Unverified Marks: 20  /  Verified: 0  /  Verified with Deductions: -30  /  Verified with Deductions &amp; Milestones: -30</v>
       </c>
       <c r="C1" s="2"/>
       <c r="D1" s="3"/>
@@ -2382,7 +2382,7 @@
       </c>
       <c r="E23" s="10"/>
       <c r="F23" s="21" t="s">
-        <v>12</v>
+        <v>214</v>
       </c>
       <c r="G23" s="22">
         <v>2</v>
@@ -2390,7 +2390,7 @@
       <c r="H23" s="10"/>
       <c r="I23" s="12">
         <f t="shared" si="9"/>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J23" s="12">
         <f t="shared" si="10"/>
@@ -2500,7 +2500,7 @@
       </c>
       <c r="E26" s="10"/>
       <c r="F26" s="21" t="s">
-        <v>12</v>
+        <v>214</v>
       </c>
       <c r="G26" s="22">
         <v>2</v>
@@ -2510,7 +2510,7 @@
       </c>
       <c r="I26" s="12">
         <f t="shared" ref="I26:I27" si="11">IF(OR(F26 = "maybe", F26 = "yes"),G26, 0)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J26" s="12">
         <f t="shared" ref="J26:J27" si="12">IF(F26 = "yes",G26, 0)</f>
@@ -7999,7 +7999,7 @@
       <c r="H170" s="10"/>
       <c r="I170" s="38">
         <f t="shared" ref="I170:K170" si="24">SUM(I4:I162)</f>
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="J170" s="12">
         <f t="shared" si="24"/>

</xml_diff>

<commit_message>
Adjust product image display and add active state to navbar links
</commit_message>
<xml_diff>
--- a/Full Stack - Ecommerce Project Marking Sheet.xlsx
+++ b/Full Stack - Ecommerce Project Marking Sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\rndev\electrostore_app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22B1ACEC-2571-45E2-BA3E-ED6C6C24A9AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4C008F7-E6E2-4F15-B8D4-808C0B21562D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1476,7 +1476,7 @@
     <row r="1" spans="1:29" ht="23.4" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="str">
         <f>"Unverified Marks: " &amp; I170 &amp; "  /  Verified: " &amp; J170 &amp; "  /  Verified with Deductions: " &amp; K170 &amp; "  /  Verified with Deductions &amp; Milestones: " &amp; L170</f>
-        <v>Unverified Marks: 20  /  Verified: 0  /  Verified with Deductions: -30  /  Verified with Deductions &amp; Milestones: -30</v>
+        <v>Unverified Marks: 30  /  Verified: 2  /  Verified with Deductions: -28  /  Verified with Deductions &amp; Milestones: -28</v>
       </c>
       <c r="C1" s="2"/>
       <c r="D1" s="3"/>
@@ -2738,7 +2738,7 @@
       </c>
       <c r="E32" s="10"/>
       <c r="F32" s="21" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="G32" s="22">
         <v>2</v>
@@ -2746,15 +2746,15 @@
       <c r="H32" s="10"/>
       <c r="I32" s="12">
         <f>IF(OR(F32 = "maybe", F32 = "yes"),G32, 0)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J32" s="12">
         <f>IF(F32 = "yes",G32, 0)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K32" s="12">
         <f>IF(F32 = "yes",G32, 0)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L32" s="18"/>
       <c r="M32" s="18"/>
@@ -2783,7 +2783,7 @@
         <v>55</v>
       </c>
       <c r="E33" s="21" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="F33" s="17"/>
       <c r="G33" s="22"/>
@@ -2821,7 +2821,7 @@
       </c>
       <c r="E34" s="10"/>
       <c r="F34" s="21" t="s">
-        <v>12</v>
+        <v>214</v>
       </c>
       <c r="G34" s="22">
         <v>4</v>
@@ -2831,7 +2831,7 @@
       </c>
       <c r="I34" s="12">
         <f>IF(OR(F34 = "maybe", F34 = "yes"),G34, 0)</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="J34" s="12">
         <f>IF(F34 = "yes",G34, 0)</f>
@@ -6123,7 +6123,7 @@
       </c>
       <c r="E120" s="10"/>
       <c r="F120" s="21" t="s">
-        <v>12</v>
+        <v>214</v>
       </c>
       <c r="G120" s="22">
         <v>4</v>
@@ -6133,7 +6133,7 @@
       </c>
       <c r="I120" s="12">
         <f>IF(OR(F120 = "maybe", F120 = "yes"),G120, 0)</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="J120" s="12">
         <f>IF(F120 = "yes",G120, 0)</f>
@@ -7999,19 +7999,19 @@
       <c r="H170" s="10"/>
       <c r="I170" s="38">
         <f t="shared" ref="I170:K170" si="24">SUM(I4:I162)</f>
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="J170" s="12">
         <f t="shared" si="24"/>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K170" s="12">
         <f t="shared" si="24"/>
-        <v>-30</v>
+        <v>-28</v>
       </c>
       <c r="L170" s="12">
         <f>CHOOSE(SUM(L165:L168)+1, MIN(60, K170) + (K170 - MIN(60, K170))/2,MIN(70, KJ170) + (K170 - MIN(70, K170))/2,MIN(80, K170) + (K170 - MIN(80, K170))/2,MIN(90, K170) + (K170 - MIN(90, K170))/2, K170)</f>
-        <v>-30</v>
+        <v>-28</v>
       </c>
       <c r="M170" s="18"/>
       <c r="N170" s="7"/>

</xml_diff>

<commit_message>
2.4: Filter the displayed products by new or recently updated
</commit_message>
<xml_diff>
--- a/Full Stack - Ecommerce Project Marking Sheet.xlsx
+++ b/Full Stack - Ecommerce Project Marking Sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\rndev\electrostore_app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4C008F7-E6E2-4F15-B8D4-808C0B21562D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01F6A04F-C33D-4FCE-A262-0C7B062C93FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="379" uniqueCount="215">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="379" uniqueCount="214">
   <si>
     <t>Confirm</t>
   </si>
@@ -722,9 +722,6 @@
   <si>
     <t>Yes Sum with Milestones</t>
   </si>
-  <si>
-    <t>Maybe</t>
-  </si>
 </sst>
 </file>
 
@@ -733,7 +730,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="19" x14ac:knownFonts="1">
+  <fonts count="20" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -839,7 +836,13 @@
     </font>
     <font>
       <sz val="14"/>
-      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color rgb="FFC00000"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -891,7 +894,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -984,6 +987,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1476,7 +1482,7 @@
     <row r="1" spans="1:29" ht="23.4" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="str">
         <f>"Unverified Marks: " &amp; I170 &amp; "  /  Verified: " &amp; J170 &amp; "  /  Verified with Deductions: " &amp; K170 &amp; "  /  Verified with Deductions &amp; Milestones: " &amp; L170</f>
-        <v>Unverified Marks: 30  /  Verified: 2  /  Verified with Deductions: -28  /  Verified with Deductions &amp; Milestones: -28</v>
+        <v>Unverified Marks: 30  /  Verified: 30  /  Verified with Deductions: 15  /  Verified with Deductions &amp; Milestones: 15</v>
       </c>
       <c r="C1" s="2"/>
       <c r="D1" s="3"/>
@@ -1600,7 +1606,7 @@
       </c>
       <c r="E4" s="10"/>
       <c r="F4" s="21" t="s">
-        <v>214</v>
+        <v>16</v>
       </c>
       <c r="G4" s="22">
         <v>2</v>
@@ -1614,11 +1620,11 @@
       </c>
       <c r="J4" s="12">
         <f t="shared" ref="J4:J5" si="1">IF(F4 = "yes",G4, 0)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K4" s="12">
         <f t="shared" ref="K4:K5" si="2">IF(F4 = "yes",G4, $M$2)</f>
-        <v>-3</v>
+        <v>2</v>
       </c>
       <c r="L4" s="18"/>
       <c r="M4" s="18"/>
@@ -1650,7 +1656,7 @@
       </c>
       <c r="E5" s="10"/>
       <c r="F5" s="21" t="s">
-        <v>214</v>
+        <v>16</v>
       </c>
       <c r="G5" s="22">
         <v>2</v>
@@ -1664,11 +1670,11 @@
       </c>
       <c r="J5" s="24">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K5" s="24">
         <f t="shared" si="2"/>
-        <v>-3</v>
+        <v>2</v>
       </c>
       <c r="L5" s="18"/>
       <c r="M5" s="18"/>
@@ -1732,7 +1738,7 @@
         <v>18</v>
       </c>
       <c r="E7" s="21" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="F7" s="17"/>
       <c r="G7" s="22"/>
@@ -1770,7 +1776,7 @@
       </c>
       <c r="E8" s="10"/>
       <c r="F8" s="21" t="s">
-        <v>214</v>
+        <v>16</v>
       </c>
       <c r="G8" s="22">
         <v>2</v>
@@ -1782,11 +1788,11 @@
       </c>
       <c r="J8" s="12">
         <f t="shared" ref="J8:J9" si="4">IF(F8 = "yes",G8, 0)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K8" s="12">
         <f t="shared" ref="K8:K9" si="5">IF(F8 = "yes",G8, 0)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L8" s="18"/>
       <c r="M8" s="18"/>
@@ -1971,7 +1977,7 @@
       </c>
       <c r="E13" s="10"/>
       <c r="F13" s="21" t="s">
-        <v>214</v>
+        <v>16</v>
       </c>
       <c r="G13" s="22">
         <v>2</v>
@@ -1983,11 +1989,11 @@
       </c>
       <c r="J13" s="12">
         <f>IF(F13 = "yes",G13, 0)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K13" s="12">
         <f>IF(F13 = "yes",G13, 0)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L13" s="18"/>
       <c r="M13" s="18"/>
@@ -2052,7 +2058,7 @@
       </c>
       <c r="E15" s="10"/>
       <c r="F15" s="21" t="s">
-        <v>214</v>
+        <v>16</v>
       </c>
       <c r="G15" s="22">
         <v>2</v>
@@ -2064,11 +2070,11 @@
       </c>
       <c r="J15" s="12">
         <f>IF(F15 = "yes",G15, 0)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K15" s="12">
         <f>IF(F15 = "yes",G15, 0)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L15" s="18"/>
       <c r="M15" s="18"/>
@@ -2097,7 +2103,7 @@
         <v>31</v>
       </c>
       <c r="E16" s="21" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="F16" s="17"/>
       <c r="G16" s="22"/>
@@ -2135,7 +2141,7 @@
       </c>
       <c r="E17" s="10"/>
       <c r="F17" s="21" t="s">
-        <v>214</v>
+        <v>16</v>
       </c>
       <c r="G17" s="22">
         <v>2</v>
@@ -2147,11 +2153,11 @@
       </c>
       <c r="J17" s="12">
         <f t="shared" ref="J17:J18" si="7">IF(F17 = "yes",G17, 0)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K17" s="12">
         <f t="shared" ref="K17:K18" si="8">IF(F17 = "yes",G17, 0)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L17" s="18"/>
       <c r="M17" s="18"/>
@@ -2183,7 +2189,7 @@
       </c>
       <c r="E18" s="10"/>
       <c r="F18" s="21" t="s">
-        <v>214</v>
+        <v>16</v>
       </c>
       <c r="G18" s="22">
         <v>2</v>
@@ -2195,11 +2201,11 @@
       </c>
       <c r="J18" s="12">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K18" s="12">
         <f t="shared" si="8"/>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L18" s="18"/>
       <c r="M18" s="18"/>
@@ -2228,7 +2234,7 @@
         <v>36</v>
       </c>
       <c r="E19" s="21" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="F19" s="17"/>
       <c r="G19" s="22"/>
@@ -2332,7 +2338,7 @@
       </c>
       <c r="E22" s="10"/>
       <c r="F22" s="21" t="s">
-        <v>214</v>
+        <v>16</v>
       </c>
       <c r="G22" s="22">
         <v>2</v>
@@ -2346,11 +2352,11 @@
       </c>
       <c r="J22" s="12">
         <f t="shared" ref="J22:J23" si="10">IF(F22 = "yes",G22, 0)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K22" s="12">
         <f>IF(F22 = "yes",G22, $M$2)</f>
-        <v>-3</v>
+        <v>2</v>
       </c>
       <c r="L22" s="18"/>
       <c r="M22" s="18"/>
@@ -2382,7 +2388,7 @@
       </c>
       <c r="E23" s="10"/>
       <c r="F23" s="21" t="s">
-        <v>214</v>
+        <v>16</v>
       </c>
       <c r="G23" s="22">
         <v>2</v>
@@ -2394,11 +2400,11 @@
       </c>
       <c r="J23" s="12">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K23" s="12">
         <f>IF(F23 = "yes",G23, 0)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L23" s="18"/>
       <c r="M23" s="18"/>
@@ -2427,7 +2433,7 @@
         <v>43</v>
       </c>
       <c r="E24" s="21" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="F24" s="17"/>
       <c r="G24" s="22"/>
@@ -2462,7 +2468,7 @@
         <v>44</v>
       </c>
       <c r="E25" s="21" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="F25" s="17"/>
       <c r="G25" s="22"/>
@@ -2500,7 +2506,7 @@
       </c>
       <c r="E26" s="10"/>
       <c r="F26" s="21" t="s">
-        <v>214</v>
+        <v>16</v>
       </c>
       <c r="G26" s="22">
         <v>2</v>
@@ -2514,11 +2520,11 @@
       </c>
       <c r="J26" s="12">
         <f t="shared" ref="J26:J27" si="12">IF(F26 = "yes",G26, 0)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K26" s="12">
         <f>IF(F26 = "yes",G26, $M$2)</f>
-        <v>-3</v>
+        <v>2</v>
       </c>
       <c r="L26" s="18"/>
       <c r="M26" s="18"/>
@@ -2550,7 +2556,7 @@
       </c>
       <c r="E27" s="10"/>
       <c r="F27" s="21" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="G27" s="22">
         <v>2</v>
@@ -2558,15 +2564,15 @@
       <c r="H27" s="10"/>
       <c r="I27" s="12">
         <f t="shared" si="11"/>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J27" s="12">
         <f t="shared" si="12"/>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K27" s="12">
         <f>IF(F27 = "yes",G27, 0)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L27" s="18"/>
       <c r="M27" s="18"/>
@@ -2630,7 +2636,7 @@
         <v>50</v>
       </c>
       <c r="E29" s="21" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="F29" s="17"/>
       <c r="G29" s="22"/>
@@ -2665,7 +2671,7 @@
         <v>51</v>
       </c>
       <c r="E30" s="21" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="F30" s="17"/>
       <c r="G30" s="22"/>
@@ -2700,7 +2706,7 @@
         <v>52</v>
       </c>
       <c r="E31" s="21" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="F31" s="17"/>
       <c r="G31" s="22"/>
@@ -2821,7 +2827,7 @@
       </c>
       <c r="E34" s="10"/>
       <c r="F34" s="21" t="s">
-        <v>214</v>
+        <v>16</v>
       </c>
       <c r="G34" s="22">
         <v>4</v>
@@ -2835,11 +2841,11 @@
       </c>
       <c r="J34" s="12">
         <f>IF(F34 = "yes",G34, 0)</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="K34" s="12">
         <f>IF(F34 = "yes",G34, $M$2)</f>
-        <v>-3</v>
+        <v>4</v>
       </c>
       <c r="L34" s="18"/>
       <c r="M34" s="18"/>
@@ -2868,7 +2874,7 @@
         <v>58</v>
       </c>
       <c r="E35" s="21" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="F35" s="17"/>
       <c r="G35" s="22"/>
@@ -2903,7 +2909,7 @@
         <v>59</v>
       </c>
       <c r="E36" s="21" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="F36" s="17"/>
       <c r="G36" s="22"/>
@@ -2938,7 +2944,7 @@
         <v>60</v>
       </c>
       <c r="E37" s="21" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="F37" s="17"/>
       <c r="G37" s="22"/>
@@ -2973,7 +2979,7 @@
         <v>61</v>
       </c>
       <c r="E38" s="21" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="F38" s="17"/>
       <c r="G38" s="22"/>
@@ -3008,7 +3014,7 @@
         <v>62</v>
       </c>
       <c r="E39" s="21" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="F39" s="17"/>
       <c r="G39" s="22"/>
@@ -3043,7 +3049,7 @@
         <v>63</v>
       </c>
       <c r="E40" s="21" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="F40" s="17"/>
       <c r="G40" s="22"/>
@@ -5829,7 +5835,7 @@
       </c>
       <c r="E113" s="10"/>
       <c r="F113" s="21" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="G113" s="22">
         <v>2</v>
@@ -5837,15 +5843,15 @@
       <c r="H113" s="10"/>
       <c r="I113" s="12">
         <f t="shared" ref="I113:I116" si="17">IF(OR(F113 = "maybe", F113 = "yes"),G113, 0)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J113" s="12">
         <f t="shared" ref="J113:J116" si="18">IF(F113 = "yes",G113, 0)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K113" s="12">
         <f t="shared" ref="K113:K116" si="19">IF(F113 = "yes",G113, 0)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L113" s="18"/>
       <c r="M113" s="18"/>
@@ -5968,7 +5974,7 @@
       <c r="C116" s="19" t="s">
         <v>154</v>
       </c>
-      <c r="D116" s="20" t="s">
+      <c r="D116" s="40" t="s">
         <v>155</v>
       </c>
       <c r="E116" s="10"/>
@@ -6123,7 +6129,7 @@
       </c>
       <c r="E120" s="10"/>
       <c r="F120" s="21" t="s">
-        <v>214</v>
+        <v>12</v>
       </c>
       <c r="G120" s="22">
         <v>4</v>
@@ -6133,7 +6139,7 @@
       </c>
       <c r="I120" s="12">
         <f>IF(OR(F120 = "maybe", F120 = "yes"),G120, 0)</f>
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="J120" s="12">
         <f>IF(F120 = "yes",G120, 0)</f>
@@ -8003,15 +8009,15 @@
       </c>
       <c r="J170" s="12">
         <f t="shared" si="24"/>
-        <v>2</v>
+        <v>30</v>
       </c>
       <c r="K170" s="12">
         <f t="shared" si="24"/>
-        <v>-28</v>
+        <v>15</v>
       </c>
       <c r="L170" s="12">
         <f>CHOOSE(SUM(L165:L168)+1, MIN(60, K170) + (K170 - MIN(60, K170))/2,MIN(70, KJ170) + (K170 - MIN(70, K170))/2,MIN(80, K170) + (K170 - MIN(80, K170))/2,MIN(90, K170) + (K170 - MIN(90, K170))/2, K170)</f>
-        <v>-28</v>
+        <v>15</v>
       </c>
       <c r="M170" s="18"/>
       <c r="N170" s="7"/>

</xml_diff>

<commit_message>
3.1.1 | 3.1.2 | 3.1.3: add various product (completed) | Edit quantity (completed) | complete checkout (wip)
</commit_message>
<xml_diff>
--- a/Full Stack - Ecommerce Project Marking Sheet.xlsx
+++ b/Full Stack - Ecommerce Project Marking Sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\rndev\electrostore_app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11E730C3-1D62-4425-BFAD-781F13515EEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{911CF0DF-75BB-4DDD-AF4D-586C2AA95DB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="379" uniqueCount="214">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="379" uniqueCount="215">
   <si>
     <t>Confirm</t>
   </si>
@@ -720,6 +720,9 @@
   <si>
     <t>Active Storage uploads are stored to Google Cloud or AWS S3.</t>
   </si>
+  <si>
+    <t>Maybe</t>
+  </si>
 </sst>
 </file>
 
@@ -728,7 +731,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="24" x14ac:knownFonts="1">
+  <fonts count="25" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -871,6 +874,13 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color theme="6" tint="-0.249977111117893"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -919,7 +929,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -1033,6 +1043,12 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="24" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1525,7 +1541,7 @@
     <row r="1" spans="1:29" ht="23.4" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="str">
         <f>"Unverified Marks: " &amp; I170 &amp; "  /  Verified: " &amp; J170 &amp; "  /  Verified with Deductions: " &amp; K170 &amp; "  /  Verified with Deductions &amp; Milestones: " &amp; L170</f>
-        <v>Unverified Marks: 30  /  Verified: 30  /  Verified with Deductions: 15  /  Verified with Deductions &amp; Milestones: 15</v>
+        <v>Unverified Marks: 40  /  Verified: 30  /  Verified with Deductions: 15  /  Verified with Deductions &amp; Milestones: 15</v>
       </c>
       <c r="C1" s="2"/>
       <c r="D1" s="3"/>
@@ -3196,7 +3212,7 @@
       </c>
       <c r="E43" s="10"/>
       <c r="F43" s="21" t="s">
-        <v>12</v>
+        <v>214</v>
       </c>
       <c r="G43" s="22">
         <v>4</v>
@@ -3206,7 +3222,7 @@
       </c>
       <c r="I43" s="12">
         <f t="shared" ref="I43:I44" si="13">IF(OR(F43 = "maybe", F43 = "yes"),G43, 0)</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="J43" s="12">
         <f t="shared" ref="J43:J44" si="14">IF(F43 = "yes",G43, 0)</f>
@@ -3246,7 +3262,7 @@
       </c>
       <c r="E44" s="10"/>
       <c r="F44" s="21" t="s">
-        <v>12</v>
+        <v>214</v>
       </c>
       <c r="G44" s="22">
         <v>4</v>
@@ -3254,7 +3270,7 @@
       <c r="H44" s="10"/>
       <c r="I44" s="12">
         <f t="shared" si="13"/>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="J44" s="12">
         <f t="shared" si="14"/>
@@ -5241,10 +5257,10 @@
     <row r="97" spans="1:29" ht="18" x14ac:dyDescent="0.35">
       <c r="A97" s="7"/>
       <c r="B97" s="7"/>
-      <c r="C97" s="44" t="s">
+      <c r="C97" s="42" t="s">
         <v>129</v>
       </c>
-      <c r="D97" s="45" t="s">
+      <c r="D97" s="43" t="s">
         <v>130</v>
       </c>
       <c r="E97" s="10"/>
@@ -5291,10 +5307,10 @@
     <row r="98" spans="1:29" ht="18" x14ac:dyDescent="0.35">
       <c r="A98" s="7"/>
       <c r="B98" s="7"/>
-      <c r="C98" s="44" t="s">
+      <c r="C98" s="42" t="s">
         <v>131</v>
       </c>
-      <c r="D98" s="45" t="s">
+      <c r="D98" s="43" t="s">
         <v>132</v>
       </c>
       <c r="E98" s="10"/>
@@ -5758,7 +5774,7 @@
       </c>
       <c r="E110" s="10"/>
       <c r="F110" s="21" t="s">
-        <v>12</v>
+        <v>214</v>
       </c>
       <c r="G110" s="22">
         <v>2</v>
@@ -5768,7 +5784,7 @@
       </c>
       <c r="I110" s="12">
         <f>IF(OR(F110 = "maybe", F110 = "yes"),G110, 0)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J110" s="12">
         <f>IF(F110 = "yes",G110, 0)</f>
@@ -5966,10 +5982,10 @@
     <row r="115" spans="1:29" ht="36" x14ac:dyDescent="0.35">
       <c r="A115" s="7"/>
       <c r="B115" s="7"/>
-      <c r="C115" s="19" t="s">
+      <c r="C115" s="47" t="s">
         <v>152</v>
       </c>
-      <c r="D115" s="20" t="s">
+      <c r="D115" s="48" t="s">
         <v>153</v>
       </c>
       <c r="E115" s="10"/>
@@ -6389,10 +6405,10 @@
     <row r="126" spans="1:29" ht="18" x14ac:dyDescent="0.35">
       <c r="A126" s="7"/>
       <c r="B126" s="7"/>
-      <c r="C126" s="19" t="s">
+      <c r="C126" s="42" t="s">
         <v>163</v>
       </c>
-      <c r="D126" s="20" t="s">
+      <c r="D126" s="43" t="s">
         <v>164</v>
       </c>
       <c r="E126" s="10"/>
@@ -8048,7 +8064,7 @@
       <c r="H170" s="10"/>
       <c r="I170" s="38">
         <f t="shared" ref="I170:K170" si="24">SUM(I4:I162)</f>
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="J170" s="12">
         <f t="shared" si="24"/>
@@ -37660,7 +37676,7 @@
       <formula>OR(E146="No", E147="No", E148="No", E149="No", E150="No")</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations disablePrompts="1" count="4">
+  <dataValidations count="4">
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="E6:E7 E10:E12 E16 E19 E24:E25 E28:E31 E33 E35:E40 E45:E47 E49:E53 E55:E58 E60:E61 E64:E66 E69:E72 E74:E75 E78:E81 E83 E87:E88 E90:E92 E94:E96 E99 E101:E103 E105:E109 E111:E112 E121:E125 E129:E130 E132:E134 E138:E140 E142:E144 E146:E150 E154:E159" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"No,Yes"</formula1>
     </dataValidation>

</xml_diff>

<commit_message>
3.1.3: Complete a checkout process after filling their shopping cart, including:
</commit_message>
<xml_diff>
--- a/Full Stack - Ecommerce Project Marking Sheet.xlsx
+++ b/Full Stack - Ecommerce Project Marking Sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\rndev\electrostore_app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{911CF0DF-75BB-4DDD-AF4D-586C2AA95DB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC0C6E7B-9254-496F-B5E2-888985C0988A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1541,7 +1541,7 @@
     <row r="1" spans="1:29" ht="23.4" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="str">
         <f>"Unverified Marks: " &amp; I170 &amp; "  /  Verified: " &amp; J170 &amp; "  /  Verified with Deductions: " &amp; K170 &amp; "  /  Verified with Deductions &amp; Milestones: " &amp; L170</f>
-        <v>Unverified Marks: 40  /  Verified: 30  /  Verified with Deductions: 15  /  Verified with Deductions &amp; Milestones: 15</v>
+        <v>Unverified Marks: 48  /  Verified: 30  /  Verified with Deductions: 15  /  Verified with Deductions &amp; Milestones: 15</v>
       </c>
       <c r="C1" s="2"/>
       <c r="D1" s="3"/>
@@ -3414,7 +3414,7 @@
       </c>
       <c r="E48" s="10"/>
       <c r="F48" s="21" t="s">
-        <v>12</v>
+        <v>214</v>
       </c>
       <c r="G48" s="22">
         <v>8</v>
@@ -3424,7 +3424,7 @@
       </c>
       <c r="I48" s="12">
         <f>IF(OR(F48 = "maybe", F48 = "yes"),G48, 0)</f>
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="J48" s="12">
         <f>IF(F48 = "yes",G48, 0)</f>
@@ -8064,7 +8064,7 @@
       <c r="H170" s="10"/>
       <c r="I170" s="38">
         <f t="shared" ref="I170:K170" si="24">SUM(I4:I162)</f>
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="J170" s="12">
         <f t="shared" si="24"/>

</xml_diff>

<commit_message>
3.1.4 | 3.1.5 | 4.2.1: signup new account | update profile/address | add validation
</commit_message>
<xml_diff>
--- a/Full Stack - Ecommerce Project Marking Sheet.xlsx
+++ b/Full Stack - Ecommerce Project Marking Sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\rndev\electrostore_app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC0C6E7B-9254-496F-B5E2-888985C0988A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9F7F874-E62B-49D8-AEA0-D48F304F9C51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1541,7 +1541,7 @@
     <row r="1" spans="1:29" ht="23.4" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="str">
         <f>"Unverified Marks: " &amp; I170 &amp; "  /  Verified: " &amp; J170 &amp; "  /  Verified with Deductions: " &amp; K170 &amp; "  /  Verified with Deductions &amp; Milestones: " &amp; L170</f>
-        <v>Unverified Marks: 48  /  Verified: 30  /  Verified with Deductions: 15  /  Verified with Deductions &amp; Milestones: 15</v>
+        <v>Unverified Marks: 60  /  Verified: 30  /  Verified with Deductions: 15  /  Verified with Deductions &amp; Milestones: 15</v>
       </c>
       <c r="C1" s="2"/>
       <c r="D1" s="3"/>
@@ -3639,7 +3639,7 @@
       </c>
       <c r="E54" s="10"/>
       <c r="F54" s="21" t="s">
-        <v>12</v>
+        <v>214</v>
       </c>
       <c r="G54" s="22">
         <v>8</v>
@@ -3647,7 +3647,7 @@
       <c r="H54" s="10"/>
       <c r="I54" s="12">
         <f>IF(OR(F54 = "maybe", F54 = "yes"),G54, 0)</f>
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="J54" s="12">
         <f>IF(F54 = "yes",G54, 0)</f>
@@ -3827,7 +3827,7 @@
       </c>
       <c r="E59" s="10"/>
       <c r="F59" s="21" t="s">
-        <v>12</v>
+        <v>214</v>
       </c>
       <c r="G59" s="22">
         <v>4</v>
@@ -3835,7 +3835,7 @@
       <c r="H59" s="10"/>
       <c r="I59" s="12">
         <f>IF(OR(F59 = "maybe", F59 = "yes"),G59, 0)</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="J59" s="12">
         <f>IF(F59 = "yes",G59, 0)</f>
@@ -8064,7 +8064,7 @@
       <c r="H170" s="10"/>
       <c r="I170" s="38">
         <f t="shared" ref="I170:K170" si="24">SUM(I4:I162)</f>
-        <v>48</v>
+        <v>60</v>
       </c>
       <c r="J170" s="12">
         <f t="shared" si="24"/>

</xml_diff>

<commit_message>
4.2.1 Add more validation to order, order_item
</commit_message>
<xml_diff>
--- a/Full Stack - Ecommerce Project Marking Sheet.xlsx
+++ b/Full Stack - Ecommerce Project Marking Sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\rndev\electrostore_app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9F7F874-E62B-49D8-AEA0-D48F304F9C51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0996C7AD-6755-4C82-A350-0FCE1DF2D5F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1541,7 +1541,7 @@
     <row r="1" spans="1:29" ht="23.4" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="str">
         <f>"Unverified Marks: " &amp; I170 &amp; "  /  Verified: " &amp; J170 &amp; "  /  Verified with Deductions: " &amp; K170 &amp; "  /  Verified with Deductions &amp; Milestones: " &amp; L170</f>
-        <v>Unverified Marks: 60  /  Verified: 30  /  Verified with Deductions: 15  /  Verified with Deductions &amp; Milestones: 15</v>
+        <v>Unverified Marks: 68  /  Verified: 28  /  Verified with Deductions: 13  /  Verified with Deductions &amp; Milestones: 13</v>
       </c>
       <c r="C1" s="2"/>
       <c r="D1" s="3"/>
@@ -2615,7 +2615,7 @@
       </c>
       <c r="E27" s="10"/>
       <c r="F27" s="21" t="s">
-        <v>16</v>
+        <v>214</v>
       </c>
       <c r="G27" s="22">
         <v>2</v>
@@ -2627,11 +2627,11 @@
       </c>
       <c r="J27" s="12">
         <f t="shared" si="12"/>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K27" s="12">
         <f>IF(F27 = "yes",G27, 0)</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L27" s="18"/>
       <c r="M27" s="18"/>
@@ -3204,10 +3204,10 @@
     <row r="43" spans="1:29" ht="18" x14ac:dyDescent="0.35">
       <c r="A43" s="7"/>
       <c r="B43" s="7"/>
-      <c r="C43" s="19" t="s">
+      <c r="C43" s="42" t="s">
         <v>65</v>
       </c>
-      <c r="D43" s="20" t="s">
+      <c r="D43" s="43" t="s">
         <v>66</v>
       </c>
       <c r="E43" s="10"/>
@@ -3254,10 +3254,10 @@
     <row r="44" spans="1:29" ht="18" x14ac:dyDescent="0.35">
       <c r="A44" s="7"/>
       <c r="B44" s="7"/>
-      <c r="C44" s="19" t="s">
+      <c r="C44" s="42" t="s">
         <v>67</v>
       </c>
-      <c r="D44" s="20" t="s">
+      <c r="D44" s="43" t="s">
         <v>68</v>
       </c>
       <c r="E44" s="10"/>
@@ -3406,10 +3406,10 @@
     <row r="48" spans="1:29" ht="18" x14ac:dyDescent="0.35">
       <c r="A48" s="7"/>
       <c r="B48" s="7"/>
-      <c r="C48" s="19" t="s">
+      <c r="C48" s="42" t="s">
         <v>72</v>
       </c>
-      <c r="D48" s="20" t="s">
+      <c r="D48" s="43" t="s">
         <v>73</v>
       </c>
       <c r="E48" s="10"/>
@@ -3631,10 +3631,10 @@
     <row r="54" spans="1:29" ht="18" x14ac:dyDescent="0.35">
       <c r="A54" s="7"/>
       <c r="B54" s="7"/>
-      <c r="C54" s="19" t="s">
+      <c r="C54" s="42" t="s">
         <v>79</v>
       </c>
-      <c r="D54" s="20" t="s">
+      <c r="D54" s="43" t="s">
         <v>80</v>
       </c>
       <c r="E54" s="10"/>
@@ -3819,10 +3819,10 @@
     <row r="59" spans="1:29" ht="18" x14ac:dyDescent="0.35">
       <c r="A59" s="7"/>
       <c r="B59" s="7"/>
-      <c r="C59" s="19" t="s">
+      <c r="C59" s="42" t="s">
         <v>85</v>
       </c>
-      <c r="D59" s="20" t="s">
+      <c r="D59" s="43" t="s">
         <v>86</v>
       </c>
       <c r="E59" s="10"/>
@@ -5265,7 +5265,7 @@
       </c>
       <c r="E97" s="10"/>
       <c r="F97" s="21" t="s">
-        <v>12</v>
+        <v>214</v>
       </c>
       <c r="G97" s="22">
         <v>2</v>
@@ -5275,7 +5275,7 @@
       </c>
       <c r="I97" s="12">
         <f t="shared" ref="I97:I98" si="15">IF(OR(F97 = "maybe", F97 = "yes"),G97, 0)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J97" s="12">
         <f t="shared" ref="J97:J98" si="16">IF(F97 = "yes",G97, 0)</f>
@@ -5315,7 +5315,7 @@
       </c>
       <c r="E98" s="10"/>
       <c r="F98" s="21" t="s">
-        <v>12</v>
+        <v>214</v>
       </c>
       <c r="G98" s="22">
         <v>2</v>
@@ -5323,7 +5323,7 @@
       <c r="H98" s="10"/>
       <c r="I98" s="12">
         <f t="shared" si="15"/>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J98" s="12">
         <f t="shared" si="16"/>
@@ -5766,10 +5766,10 @@
     <row r="110" spans="1:29" ht="36" x14ac:dyDescent="0.35">
       <c r="A110" s="7"/>
       <c r="B110" s="7"/>
-      <c r="C110" s="19" t="s">
+      <c r="C110" s="42" t="s">
         <v>144</v>
       </c>
-      <c r="D110" s="20" t="s">
+      <c r="D110" s="43" t="s">
         <v>145</v>
       </c>
       <c r="E110" s="10"/>
@@ -6413,7 +6413,7 @@
       </c>
       <c r="E126" s="10"/>
       <c r="F126" s="21" t="s">
-        <v>12</v>
+        <v>214</v>
       </c>
       <c r="G126" s="22">
         <v>4</v>
@@ -6421,7 +6421,7 @@
       <c r="H126" s="10"/>
       <c r="I126" s="12">
         <f t="shared" ref="I126:I128" si="20">IF(OR(F126 = "maybe", F126 = "yes"),G126, 0)</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="J126" s="12">
         <f t="shared" ref="J126:J128" si="21">IF(F126 = "yes",G126, 0)</f>
@@ -8064,19 +8064,19 @@
       <c r="H170" s="10"/>
       <c r="I170" s="38">
         <f t="shared" ref="I170:K170" si="24">SUM(I4:I162)</f>
-        <v>60</v>
+        <v>68</v>
       </c>
       <c r="J170" s="12">
         <f t="shared" si="24"/>
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="K170" s="12">
         <f t="shared" si="24"/>
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="L170" s="12">
         <f>CHOOSE(SUM(L165:L168)+1, MIN(60, K170) + (K170 - MIN(60, K170))/2,MIN(70, KJ170) + (K170 - MIN(70, K170))/2,MIN(80, K170) + (K170 - MIN(80, K170))/2,MIN(90, K170) + (K170 - MIN(90, K170))/2, K170)</f>
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="M170" s="18"/>
       <c r="N170" s="7"/>

</xml_diff>

<commit_message>
Change label HST to HST/GST on invoice
</commit_message>
<xml_diff>
--- a/Full Stack - Ecommerce Project Marking Sheet.xlsx
+++ b/Full Stack - Ecommerce Project Marking Sheet.xlsx
@@ -8,13 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\rndev\electrostore_app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0996C7AD-6755-4C82-A350-0FCE1DF2D5F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AD55A29-21EC-49F5-B90F-A0805221EE49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$AC$1119</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -37516,6 +37519,7 @@
       <c r="AC1119" s="7"/>
     </row>
   </sheetData>
+  <autoFilter ref="A1:AC1119" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <conditionalFormatting sqref="A4:D4">
     <cfRule type="expression" dxfId="31" priority="32">
       <formula>F4 = "Yes"</formula>

</xml_diff>

<commit_message>
3.2.1 | 3.3.1 | 3.3.2: List past orders | Integrate Stripe | Changes to product prices not affecting Past orders
</commit_message>
<xml_diff>
--- a/Full Stack - Ecommerce Project Marking Sheet.xlsx
+++ b/Full Stack - Ecommerce Project Marking Sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\rndev\electrostore_app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AD55A29-21EC-49F5-B90F-A0805221EE49}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5DF16850-8099-44FB-810D-5B95E4CD77D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="379" uniqueCount="215">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="379" uniqueCount="214">
   <si>
     <t>Confirm</t>
   </si>
@@ -723,9 +723,6 @@
   <si>
     <t>Active Storage uploads are stored to Google Cloud or AWS S3.</t>
   </si>
-  <si>
-    <t>Maybe</t>
-  </si>
 </sst>
 </file>
 
@@ -734,7 +731,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="25" x14ac:knownFonts="1">
+  <fonts count="23" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -852,40 +849,25 @@
     <font>
       <b/>
       <sz val="14"/>
-      <color rgb="FFC00000"/>
+      <color theme="6" tint="-0.249977111117893"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="14"/>
-      <color rgb="FF434343"/>
+      <color rgb="FFFFC000"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="14"/>
-      <color rgb="FF00B050"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="14"/>
-      <color theme="8" tint="0.39997558519241921"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="14"/>
-      <color theme="6" tint="-0.249977111117893"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -902,6 +884,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFFFF"/>
         <bgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B050"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -932,7 +920,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -1027,31 +1015,19 @@
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="22" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="23" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="24" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1544,7 +1520,7 @@
     <row r="1" spans="1:29" ht="23.4" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="str">
         <f>"Unverified Marks: " &amp; I170 &amp; "  /  Verified: " &amp; J170 &amp; "  /  Verified with Deductions: " &amp; K170 &amp; "  /  Verified with Deductions &amp; Milestones: " &amp; L170</f>
-        <v>Unverified Marks: 68  /  Verified: 28  /  Verified with Deductions: 13  /  Verified with Deductions &amp; Milestones: 13</v>
+        <v>Unverified Marks: 70  /  Verified: 70  /  Verified with Deductions: 67  /  Verified with Deductions &amp; Milestones: 63.5</v>
       </c>
       <c r="C1" s="2"/>
       <c r="D1" s="3"/>
@@ -2610,15 +2586,15 @@
     <row r="27" spans="1:29" ht="18" x14ac:dyDescent="0.35">
       <c r="A27" s="9"/>
       <c r="B27" s="9"/>
-      <c r="C27" s="42" t="s">
+      <c r="C27" s="19" t="s">
         <v>47</v>
       </c>
-      <c r="D27" s="43" t="s">
+      <c r="D27" s="20" t="s">
         <v>48</v>
       </c>
       <c r="E27" s="10"/>
       <c r="F27" s="21" t="s">
-        <v>214</v>
+        <v>16</v>
       </c>
       <c r="G27" s="22">
         <v>2</v>
@@ -2630,11 +2606,11 @@
       </c>
       <c r="J27" s="12">
         <f t="shared" si="12"/>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K27" s="12">
         <f>IF(F27 = "yes",G27, 0)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L27" s="18"/>
       <c r="M27" s="18"/>
@@ -3207,15 +3183,15 @@
     <row r="43" spans="1:29" ht="18" x14ac:dyDescent="0.35">
       <c r="A43" s="7"/>
       <c r="B43" s="7"/>
-      <c r="C43" s="42" t="s">
+      <c r="C43" s="19" t="s">
         <v>65</v>
       </c>
-      <c r="D43" s="43" t="s">
+      <c r="D43" s="20" t="s">
         <v>66</v>
       </c>
       <c r="E43" s="10"/>
       <c r="F43" s="21" t="s">
-        <v>214</v>
+        <v>16</v>
       </c>
       <c r="G43" s="22">
         <v>4</v>
@@ -3229,11 +3205,11 @@
       </c>
       <c r="J43" s="12">
         <f t="shared" ref="J43:J44" si="14">IF(F43 = "yes",G43, 0)</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="K43" s="12">
         <f>IF(F43 = "yes",G43, $M$2)</f>
-        <v>-3</v>
+        <v>4</v>
       </c>
       <c r="L43" s="18"/>
       <c r="M43" s="18"/>
@@ -3257,15 +3233,15 @@
     <row r="44" spans="1:29" ht="18" x14ac:dyDescent="0.35">
       <c r="A44" s="7"/>
       <c r="B44" s="7"/>
-      <c r="C44" s="42" t="s">
+      <c r="C44" s="19" t="s">
         <v>67</v>
       </c>
-      <c r="D44" s="43" t="s">
+      <c r="D44" s="20" t="s">
         <v>68</v>
       </c>
       <c r="E44" s="10"/>
       <c r="F44" s="21" t="s">
-        <v>214</v>
+        <v>16</v>
       </c>
       <c r="G44" s="22">
         <v>4</v>
@@ -3277,11 +3253,11 @@
       </c>
       <c r="J44" s="12">
         <f t="shared" si="14"/>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="K44" s="12">
         <f>IF(F44 = "yes",G44, 0)</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="L44" s="18"/>
       <c r="M44" s="18"/>
@@ -3309,7 +3285,7 @@
         <v>69</v>
       </c>
       <c r="E45" s="26" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="F45" s="17"/>
       <c r="G45" s="22"/>
@@ -3344,7 +3320,7 @@
         <v>70</v>
       </c>
       <c r="E46" s="26" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="F46" s="17"/>
       <c r="G46" s="22"/>
@@ -3379,7 +3355,7 @@
         <v>71</v>
       </c>
       <c r="E47" s="26" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="F47" s="17"/>
       <c r="G47" s="22"/>
@@ -3409,15 +3385,15 @@
     <row r="48" spans="1:29" ht="18" x14ac:dyDescent="0.35">
       <c r="A48" s="7"/>
       <c r="B48" s="7"/>
-      <c r="C48" s="42" t="s">
+      <c r="C48" s="19" t="s">
         <v>72</v>
       </c>
-      <c r="D48" s="43" t="s">
+      <c r="D48" s="20" t="s">
         <v>73</v>
       </c>
       <c r="E48" s="10"/>
       <c r="F48" s="21" t="s">
-        <v>214</v>
+        <v>16</v>
       </c>
       <c r="G48" s="22">
         <v>8</v>
@@ -3431,11 +3407,11 @@
       </c>
       <c r="J48" s="12">
         <f>IF(F48 = "yes",G48, 0)</f>
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="K48" s="12">
         <f>IF(F48 = "yes",G48, $M$2)</f>
-        <v>-3</v>
+        <v>8</v>
       </c>
       <c r="L48" s="18"/>
       <c r="M48" s="18"/>
@@ -3464,7 +3440,7 @@
         <v>74</v>
       </c>
       <c r="E49" s="21" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="F49" s="17"/>
       <c r="G49" s="22"/>
@@ -3499,7 +3475,7 @@
         <v>75</v>
       </c>
       <c r="E50" s="21" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="F50" s="17"/>
       <c r="G50" s="22"/>
@@ -3534,7 +3510,7 @@
         <v>76</v>
       </c>
       <c r="E51" s="21" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="F51" s="17"/>
       <c r="G51" s="22"/>
@@ -3569,7 +3545,7 @@
         <v>77</v>
       </c>
       <c r="E52" s="21" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="F52" s="17"/>
       <c r="G52" s="22"/>
@@ -3604,7 +3580,7 @@
         <v>78</v>
       </c>
       <c r="E53" s="21" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="F53" s="17"/>
       <c r="G53" s="22"/>
@@ -3634,15 +3610,15 @@
     <row r="54" spans="1:29" ht="18" x14ac:dyDescent="0.35">
       <c r="A54" s="7"/>
       <c r="B54" s="7"/>
-      <c r="C54" s="42" t="s">
+      <c r="C54" s="19" t="s">
         <v>79</v>
       </c>
-      <c r="D54" s="43" t="s">
+      <c r="D54" s="20" t="s">
         <v>80</v>
       </c>
       <c r="E54" s="10"/>
       <c r="F54" s="21" t="s">
-        <v>214</v>
+        <v>16</v>
       </c>
       <c r="G54" s="22">
         <v>8</v>
@@ -3654,11 +3630,11 @@
       </c>
       <c r="J54" s="12">
         <f>IF(F54 = "yes",G54, 0)</f>
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="K54" s="12">
         <f>IF(F54 = "yes",G54, 0)</f>
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="L54" s="18"/>
       <c r="M54" s="18"/>
@@ -3687,7 +3663,7 @@
         <v>81</v>
       </c>
       <c r="E55" s="21" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="F55" s="17"/>
       <c r="G55" s="22"/>
@@ -3722,7 +3698,7 @@
         <v>82</v>
       </c>
       <c r="E56" s="21" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="F56" s="17"/>
       <c r="G56" s="22"/>
@@ -3757,7 +3733,7 @@
         <v>83</v>
       </c>
       <c r="E57" s="21" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="F57" s="17"/>
       <c r="G57" s="22"/>
@@ -3792,7 +3768,7 @@
         <v>84</v>
       </c>
       <c r="E58" s="21" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="F58" s="17"/>
       <c r="G58" s="22"/>
@@ -3822,15 +3798,15 @@
     <row r="59" spans="1:29" ht="18" x14ac:dyDescent="0.35">
       <c r="A59" s="7"/>
       <c r="B59" s="7"/>
-      <c r="C59" s="42" t="s">
+      <c r="C59" s="19" t="s">
         <v>85</v>
       </c>
-      <c r="D59" s="43" t="s">
+      <c r="D59" s="20" t="s">
         <v>86</v>
       </c>
       <c r="E59" s="10"/>
       <c r="F59" s="21" t="s">
-        <v>214</v>
+        <v>16</v>
       </c>
       <c r="G59" s="22">
         <v>4</v>
@@ -3842,11 +3818,11 @@
       </c>
       <c r="J59" s="12">
         <f>IF(F59 = "yes",G59, 0)</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="K59" s="12">
         <f>IF(F59 = "yes",G59, 0)</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="L59" s="18"/>
       <c r="M59" s="18"/>
@@ -3875,7 +3851,7 @@
         <v>87</v>
       </c>
       <c r="E60" s="21" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="F60" s="17"/>
       <c r="G60" s="17"/>
@@ -3910,7 +3886,7 @@
         <v>88</v>
       </c>
       <c r="E61" s="21" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="F61" s="17"/>
       <c r="G61" s="17"/>
@@ -3976,7 +3952,7 @@
       <c r="C63" s="19" t="s">
         <v>90</v>
       </c>
-      <c r="D63" s="20" t="s">
+      <c r="D63" s="44" t="s">
         <v>91</v>
       </c>
       <c r="E63" s="10"/>
@@ -4162,7 +4138,7 @@
       <c r="C68" s="19" t="s">
         <v>96</v>
       </c>
-      <c r="D68" s="20" t="s">
+      <c r="D68" s="44" t="s">
         <v>97</v>
       </c>
       <c r="E68" s="10"/>
@@ -4350,7 +4326,7 @@
       <c r="C73" s="19" t="s">
         <v>102</v>
       </c>
-      <c r="D73" s="20" t="s">
+      <c r="D73" s="44" t="s">
         <v>103</v>
       </c>
       <c r="E73" s="10"/>
@@ -4501,7 +4477,7 @@
       <c r="C77" s="19" t="s">
         <v>106</v>
       </c>
-      <c r="D77" s="20" t="s">
+      <c r="D77" s="44" t="s">
         <v>107</v>
       </c>
       <c r="E77" s="10"/>
@@ -4686,10 +4662,10 @@
     <row r="82" spans="1:29" ht="18" x14ac:dyDescent="0.35">
       <c r="A82" s="7"/>
       <c r="B82" s="7"/>
-      <c r="C82" s="44" t="s">
+      <c r="C82" s="19" t="s">
         <v>112</v>
       </c>
-      <c r="D82" s="45" t="s">
+      <c r="D82" s="44" t="s">
         <v>113</v>
       </c>
       <c r="E82" s="10"/>
@@ -4956,7 +4932,7 @@
       <c r="C89" s="19" t="s">
         <v>121</v>
       </c>
-      <c r="D89" s="20" t="s">
+      <c r="D89" s="44" t="s">
         <v>122</v>
       </c>
       <c r="E89" s="10"/>
@@ -5260,15 +5236,15 @@
     <row r="97" spans="1:29" ht="18" x14ac:dyDescent="0.35">
       <c r="A97" s="7"/>
       <c r="B97" s="7"/>
-      <c r="C97" s="42" t="s">
+      <c r="C97" s="19" t="s">
         <v>129</v>
       </c>
-      <c r="D97" s="43" t="s">
+      <c r="D97" s="20" t="s">
         <v>130</v>
       </c>
       <c r="E97" s="10"/>
       <c r="F97" s="21" t="s">
-        <v>214</v>
+        <v>16</v>
       </c>
       <c r="G97" s="22">
         <v>2</v>
@@ -5282,11 +5258,11 @@
       </c>
       <c r="J97" s="12">
         <f t="shared" ref="J97:J98" si="16">IF(F97 = "yes",G97, 0)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K97" s="12">
         <f>IF(F97 = "yes",G97, $M$2)</f>
-        <v>-3</v>
+        <v>2</v>
       </c>
       <c r="L97" s="18"/>
       <c r="M97" s="18"/>
@@ -5310,15 +5286,15 @@
     <row r="98" spans="1:29" ht="18" x14ac:dyDescent="0.35">
       <c r="A98" s="7"/>
       <c r="B98" s="7"/>
-      <c r="C98" s="42" t="s">
+      <c r="C98" s="19" t="s">
         <v>131</v>
       </c>
-      <c r="D98" s="43" t="s">
+      <c r="D98" s="20" t="s">
         <v>132</v>
       </c>
       <c r="E98" s="10"/>
       <c r="F98" s="21" t="s">
-        <v>214</v>
+        <v>16</v>
       </c>
       <c r="G98" s="22">
         <v>2</v>
@@ -5330,11 +5306,11 @@
       </c>
       <c r="J98" s="12">
         <f t="shared" si="16"/>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K98" s="12">
         <f>IF(F98 = "yes",G98, 0)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L98" s="18"/>
       <c r="M98" s="18"/>
@@ -5396,7 +5372,7 @@
       <c r="C100" s="19" t="s">
         <v>134</v>
       </c>
-      <c r="D100" s="20" t="s">
+      <c r="D100" s="44" t="s">
         <v>135</v>
       </c>
       <c r="E100" s="10"/>
@@ -5769,15 +5745,15 @@
     <row r="110" spans="1:29" ht="36" x14ac:dyDescent="0.35">
       <c r="A110" s="7"/>
       <c r="B110" s="7"/>
-      <c r="C110" s="42" t="s">
+      <c r="C110" s="19" t="s">
         <v>144</v>
       </c>
-      <c r="D110" s="43" t="s">
+      <c r="D110" s="20" t="s">
         <v>145</v>
       </c>
       <c r="E110" s="10"/>
       <c r="F110" s="21" t="s">
-        <v>214</v>
+        <v>16</v>
       </c>
       <c r="G110" s="22">
         <v>2</v>
@@ -5791,11 +5767,11 @@
       </c>
       <c r="J110" s="12">
         <f>IF(F110 = "yes",G110, 0)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K110" s="12">
         <f>IF(F110 = "yes",G110, $M$2)</f>
-        <v>-3</v>
+        <v>2</v>
       </c>
       <c r="L110" s="18"/>
       <c r="M110" s="18"/>
@@ -5985,10 +5961,10 @@
     <row r="115" spans="1:29" ht="36" x14ac:dyDescent="0.35">
       <c r="A115" s="7"/>
       <c r="B115" s="7"/>
-      <c r="C115" s="47" t="s">
+      <c r="C115" s="41" t="s">
         <v>152</v>
       </c>
-      <c r="D115" s="48" t="s">
+      <c r="D115" s="42" t="s">
         <v>153</v>
       </c>
       <c r="E115" s="10"/>
@@ -6036,12 +6012,12 @@
       <c r="C116" s="19" t="s">
         <v>154</v>
       </c>
-      <c r="D116" s="40" t="s">
+      <c r="D116" s="20" t="s">
         <v>155</v>
       </c>
       <c r="E116" s="10"/>
       <c r="F116" s="21" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="G116" s="22">
         <v>2</v>
@@ -6049,15 +6025,15 @@
       <c r="H116" s="10"/>
       <c r="I116" s="12">
         <f t="shared" si="17"/>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J116" s="12">
         <f t="shared" si="18"/>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K116" s="12">
         <f t="shared" si="19"/>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L116" s="18"/>
       <c r="M116" s="18"/>
@@ -6186,7 +6162,7 @@
       <c r="C120" s="19" t="s">
         <v>157</v>
       </c>
-      <c r="D120" s="20" t="s">
+      <c r="D120" s="44" t="s">
         <v>158</v>
       </c>
       <c r="E120" s="10"/>
@@ -6374,7 +6350,7 @@
       <c r="A125" s="7"/>
       <c r="B125" s="7"/>
       <c r="C125" s="19"/>
-      <c r="D125" s="46" t="s">
+      <c r="D125" s="40" t="s">
         <v>212</v>
       </c>
       <c r="E125" s="21" t="s">
@@ -6408,15 +6384,15 @@
     <row r="126" spans="1:29" ht="18" x14ac:dyDescent="0.35">
       <c r="A126" s="7"/>
       <c r="B126" s="7"/>
-      <c r="C126" s="42" t="s">
+      <c r="C126" s="19" t="s">
         <v>163</v>
       </c>
-      <c r="D126" s="43" t="s">
+      <c r="D126" s="20" t="s">
         <v>164</v>
       </c>
       <c r="E126" s="10"/>
       <c r="F126" s="21" t="s">
-        <v>214</v>
+        <v>16</v>
       </c>
       <c r="G126" s="22">
         <v>4</v>
@@ -6428,11 +6404,11 @@
       </c>
       <c r="J126" s="12">
         <f t="shared" ref="J126:J128" si="21">IF(F126 = "yes",G126, 0)</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="K126" s="12">
         <f t="shared" ref="K126:K128" si="22">IF(F126 = "yes",G126, 0)</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="L126" s="18"/>
       <c r="M126" s="18"/>
@@ -6459,7 +6435,7 @@
       <c r="C127" s="19" t="s">
         <v>165</v>
       </c>
-      <c r="D127" s="41" t="s">
+      <c r="D127" s="44" t="s">
         <v>213</v>
       </c>
       <c r="E127" s="10"/>
@@ -6989,7 +6965,7 @@
       <c r="C141" s="19" t="s">
         <v>180</v>
       </c>
-      <c r="D141" s="20" t="s">
+      <c r="D141" s="43" t="s">
         <v>181</v>
       </c>
       <c r="E141" s="7"/>
@@ -7142,7 +7118,7 @@
       <c r="C145" s="19" t="s">
         <v>183</v>
       </c>
-      <c r="D145" s="20" t="s">
+      <c r="D145" s="43" t="s">
         <v>184</v>
       </c>
       <c r="E145" s="10"/>
@@ -8067,19 +8043,19 @@
       <c r="H170" s="10"/>
       <c r="I170" s="38">
         <f t="shared" ref="I170:K170" si="24">SUM(I4:I162)</f>
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="J170" s="12">
         <f t="shared" si="24"/>
-        <v>28</v>
+        <v>70</v>
       </c>
       <c r="K170" s="12">
         <f t="shared" si="24"/>
-        <v>13</v>
+        <v>67</v>
       </c>
       <c r="L170" s="12">
         <f>CHOOSE(SUM(L165:L168)+1, MIN(60, K170) + (K170 - MIN(60, K170))/2,MIN(70, KJ170) + (K170 - MIN(70, K170))/2,MIN(80, K170) + (K170 - MIN(80, K170))/2,MIN(90, K170) + (K170 - MIN(90, K170))/2, K170)</f>
-        <v>13</v>
+        <v>63.5</v>
       </c>
       <c r="M170" s="18"/>
       <c r="N170" s="7"/>
@@ -37680,8 +37656,8 @@
       <formula>OR(E146="No", E147="No", E148="No", E149="No", E150="No")</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="4">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="E6:E7 E10:E12 E16 E19 E24:E25 E28:E31 E33 E35:E40 E45:E47 E49:E53 E55:E58 E60:E61 E64:E66 E69:E72 E74:E75 E78:E81 E83 E87:E88 E90:E92 E94:E96 E99 E101:E103 E105:E109 E111:E112 E121:E125 E129:E130 E132:E134 E138:E140 E142:E144 E146:E150 E154:E159" xr:uid="{00000000-0002-0000-0000-000000000000}">
+  <dataValidations disablePrompts="1" count="4">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="E6:E7 E10:E12 E16 E19 E24:E25 E28:E31 E33 E35:E40 E45:E47 E154:E159 E49:E53 E55:E58 E64:E66 E69:E72 E74:E75 E78:E81 E83 E87:E88 E90:E92 E94:E96 E99 E101:E103 E105:E109 E111:E112 E121:E125 E129:E130 E132:E134 E138:E140 E142:E144 E146:E150 E60:E61" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"No,Yes"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="F153 F162" xr:uid="{00000000-0002-0000-0000-000001000000}">

</xml_diff>

<commit_message>
3.2.2: Admin can change status of an order
</commit_message>
<xml_diff>
--- a/Full Stack - Ecommerce Project Marking Sheet.xlsx
+++ b/Full Stack - Ecommerce Project Marking Sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\rndev\electrostore_app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5DF16850-8099-44FB-810D-5B95E4CD77D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5F0B907-E2F3-4AA1-A7E7-D36B12C5DAAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="379" uniqueCount="214">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="379" uniqueCount="215">
   <si>
     <t>Confirm</t>
   </si>
@@ -723,6 +723,9 @@
   <si>
     <t>Active Storage uploads are stored to Google Cloud or AWS S3.</t>
   </si>
+  <si>
+    <t>Maybe</t>
+  </si>
 </sst>
 </file>
 
@@ -867,7 +870,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -889,6 +892,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF00B050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -920,7 +929,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="46">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -1028,6 +1037,9 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1520,7 +1532,7 @@
     <row r="1" spans="1:29" ht="23.4" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="str">
         <f>"Unverified Marks: " &amp; I170 &amp; "  /  Verified: " &amp; J170 &amp; "  /  Verified with Deductions: " &amp; K170 &amp; "  /  Verified with Deductions &amp; Milestones: " &amp; L170</f>
-        <v>Unverified Marks: 70  /  Verified: 70  /  Verified with Deductions: 67  /  Verified with Deductions &amp; Milestones: 63.5</v>
+        <v>Unverified Marks: 84  /  Verified: 70  /  Verified with Deductions: 67  /  Verified with Deductions &amp; Milestones: 63.5</v>
       </c>
       <c r="C1" s="2"/>
       <c r="D1" s="3"/>
@@ -3952,12 +3964,12 @@
       <c r="C63" s="19" t="s">
         <v>90</v>
       </c>
-      <c r="D63" s="44" t="s">
+      <c r="D63" s="45" t="s">
         <v>91</v>
       </c>
       <c r="E63" s="10"/>
       <c r="F63" s="21" t="s">
-        <v>12</v>
+        <v>214</v>
       </c>
       <c r="G63" s="22">
         <v>4</v>
@@ -3965,7 +3977,7 @@
       <c r="H63" s="10"/>
       <c r="I63" s="12">
         <f>IF(OR(F63 = "maybe", F63 = "yes"),G63, 0)</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="J63" s="12">
         <f>IF(F63 = "yes",G63, 0)</f>
@@ -4002,7 +4014,7 @@
         <v>92</v>
       </c>
       <c r="E64" s="21" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="F64" s="17"/>
       <c r="G64" s="22"/>
@@ -4138,12 +4150,12 @@
       <c r="C68" s="19" t="s">
         <v>96</v>
       </c>
-      <c r="D68" s="44" t="s">
+      <c r="D68" s="45" t="s">
         <v>97</v>
       </c>
       <c r="E68" s="10"/>
       <c r="F68" s="21" t="s">
-        <v>12</v>
+        <v>214</v>
       </c>
       <c r="G68" s="22">
         <v>2</v>
@@ -4151,7 +4163,7 @@
       <c r="H68" s="10"/>
       <c r="I68" s="12">
         <f>IF(OR(F68 = "maybe", F68 = "yes"),G68, 0)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J68" s="12">
         <f>IF(F68 = "yes",G68, 0)</f>
@@ -4188,7 +4200,7 @@
         <v>98</v>
       </c>
       <c r="E69" s="21" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="F69" s="17"/>
       <c r="G69" s="22"/>
@@ -4223,7 +4235,7 @@
         <v>99</v>
       </c>
       <c r="E70" s="21" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="F70" s="17"/>
       <c r="G70" s="22"/>
@@ -4258,7 +4270,7 @@
         <v>100</v>
       </c>
       <c r="E71" s="21" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="F71" s="17"/>
       <c r="G71" s="22"/>
@@ -4293,7 +4305,7 @@
         <v>101</v>
       </c>
       <c r="E72" s="21" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="F72" s="17"/>
       <c r="G72" s="22"/>
@@ -4477,12 +4489,12 @@
       <c r="C77" s="19" t="s">
         <v>106</v>
       </c>
-      <c r="D77" s="44" t="s">
+      <c r="D77" s="45" t="s">
         <v>107</v>
       </c>
       <c r="E77" s="10"/>
       <c r="F77" s="21" t="s">
-        <v>12</v>
+        <v>214</v>
       </c>
       <c r="G77" s="22">
         <v>6</v>
@@ -4490,7 +4502,7 @@
       <c r="H77" s="10"/>
       <c r="I77" s="12">
         <f>IF(OR(F77 = "maybe", F77 = "yes"),G77, 0)</f>
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="J77" s="12">
         <f>IF(F77 = "yes",G77, 0)</f>
@@ -4527,7 +4539,7 @@
         <v>108</v>
       </c>
       <c r="E78" s="21" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="F78" s="17"/>
       <c r="G78" s="22"/>
@@ -4562,7 +4574,7 @@
         <v>109</v>
       </c>
       <c r="E79" s="21" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="F79" s="17"/>
       <c r="G79" s="22"/>
@@ -4597,7 +4609,7 @@
         <v>110</v>
       </c>
       <c r="E80" s="21" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="F80" s="17"/>
       <c r="G80" s="22"/>
@@ -4632,7 +4644,7 @@
         <v>111</v>
       </c>
       <c r="E81" s="21" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="F81" s="17"/>
       <c r="G81" s="22"/>
@@ -4665,12 +4677,12 @@
       <c r="C82" s="19" t="s">
         <v>112</v>
       </c>
-      <c r="D82" s="44" t="s">
+      <c r="D82" s="45" t="s">
         <v>113</v>
       </c>
       <c r="E82" s="10"/>
       <c r="F82" s="21" t="s">
-        <v>12</v>
+        <v>214</v>
       </c>
       <c r="G82" s="22">
         <v>2</v>
@@ -4678,7 +4690,7 @@
       <c r="H82" s="10"/>
       <c r="I82" s="12">
         <f>IF(OR(F82 = "maybe", F82 = "yes"),G82, 0)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J82" s="12">
         <f>IF(F82 = "yes",G82, 0)</f>
@@ -4715,7 +4727,7 @@
         <v>114</v>
       </c>
       <c r="E83" s="21" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="F83" s="17"/>
       <c r="G83" s="22"/>
@@ -8043,7 +8055,7 @@
       <c r="H170" s="10"/>
       <c r="I170" s="38">
         <f t="shared" ref="I170:K170" si="24">SUM(I4:I162)</f>
-        <v>70</v>
+        <v>84</v>
       </c>
       <c r="J170" s="12">
         <f t="shared" si="24"/>
@@ -37656,7 +37668,7 @@
       <formula>OR(E146="No", E147="No", E148="No", E149="No", E150="No")</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations disablePrompts="1" count="4">
+  <dataValidations count="4">
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="E6:E7 E10:E12 E16 E19 E24:E25 E28:E31 E33 E35:E40 E45:E47 E154:E159 E49:E53 E55:E58 E64:E66 E69:E72 E74:E75 E78:E81 E83 E87:E88 E90:E92 E94:E96 E99 E101:E103 E105:E109 E111:E112 E121:E125 E129:E130 E132:E134 E138:E140 E142:E144 E146:E150 E60:E61" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"No,Yes"</formula1>
     </dataValidation>

</xml_diff>

<commit_message>
5.3: Active Storage uploads are stored to AWS S3
</commit_message>
<xml_diff>
--- a/Full Stack - Ecommerce Project Marking Sheet.xlsx
+++ b/Full Stack - Ecommerce Project Marking Sheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\rndev\electrostore_app\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5F0B907-E2F3-4AA1-A7E7-D36B12C5DAAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{652E65FB-1E57-4526-B467-CA60B2AE1405}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -870,7 +870,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -887,12 +887,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFFFF"/>
         <bgColor rgb="FFFFFFFF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF00B050"/>
-        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
@@ -929,7 +923,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -1037,9 +1031,6 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1532,7 +1523,7 @@
     <row r="1" spans="1:29" ht="23.4" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="str">
         <f>"Unverified Marks: " &amp; I170 &amp; "  /  Verified: " &amp; J170 &amp; "  /  Verified with Deductions: " &amp; K170 &amp; "  /  Verified with Deductions &amp; Milestones: " &amp; L170</f>
-        <v>Unverified Marks: 84  /  Verified: 70  /  Verified with Deductions: 67  /  Verified with Deductions &amp; Milestones: 63.5</v>
+        <v>Unverified Marks: 96  /  Verified: 78  /  Verified with Deductions: 78  /  Verified with Deductions &amp; Milestones: 69</v>
       </c>
       <c r="C1" s="2"/>
       <c r="D1" s="3"/>
@@ -3964,7 +3955,7 @@
       <c r="C63" s="19" t="s">
         <v>90</v>
       </c>
-      <c r="D63" s="45" t="s">
+      <c r="D63" s="44" t="s">
         <v>91</v>
       </c>
       <c r="E63" s="10"/>
@@ -4150,7 +4141,7 @@
       <c r="C68" s="19" t="s">
         <v>96</v>
       </c>
-      <c r="D68" s="45" t="s">
+      <c r="D68" s="44" t="s">
         <v>97</v>
       </c>
       <c r="E68" s="10"/>
@@ -4343,7 +4334,7 @@
       </c>
       <c r="E73" s="10"/>
       <c r="F73" s="21" t="s">
-        <v>12</v>
+        <v>214</v>
       </c>
       <c r="G73" s="22">
         <v>2</v>
@@ -4351,7 +4342,7 @@
       <c r="H73" s="10"/>
       <c r="I73" s="12">
         <f>IF(OR(F73 = "maybe", F73 = "yes"),G73, 0)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J73" s="12">
         <f>IF(F73 = "yes",G73, 0)</f>
@@ -4489,7 +4480,7 @@
       <c r="C77" s="19" t="s">
         <v>106</v>
       </c>
-      <c r="D77" s="45" t="s">
+      <c r="D77" s="44" t="s">
         <v>107</v>
       </c>
       <c r="E77" s="10"/>
@@ -4677,7 +4668,7 @@
       <c r="C82" s="19" t="s">
         <v>112</v>
       </c>
-      <c r="D82" s="45" t="s">
+      <c r="D82" s="44" t="s">
         <v>113</v>
       </c>
       <c r="E82" s="10"/>
@@ -5389,7 +5380,7 @@
       </c>
       <c r="E100" s="10"/>
       <c r="F100" s="21" t="s">
-        <v>12</v>
+        <v>214</v>
       </c>
       <c r="G100" s="22">
         <v>2</v>
@@ -5397,7 +5388,7 @@
       <c r="H100" s="10"/>
       <c r="I100" s="12">
         <f>IF(OR(F100 = "maybe", F100 = "yes"),G100, 0)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J100" s="12">
         <f>IF(F100 = "yes",G100, 0)</f>
@@ -6179,7 +6170,7 @@
       </c>
       <c r="E120" s="10"/>
       <c r="F120" s="21" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="G120" s="22">
         <v>4</v>
@@ -6189,15 +6180,15 @@
       </c>
       <c r="I120" s="12">
         <f>IF(OR(F120 = "maybe", F120 = "yes"),G120, 0)</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="J120" s="12">
         <f>IF(F120 = "yes",G120, 0)</f>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="K120" s="12">
         <f>IF(F120 = "yes",G120, $M$2)</f>
-        <v>-3</v>
+        <v>4</v>
       </c>
       <c r="L120" s="18"/>
       <c r="M120" s="18"/>
@@ -6226,7 +6217,7 @@
         <v>159</v>
       </c>
       <c r="E121" s="21" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="F121" s="17"/>
       <c r="G121" s="22"/>
@@ -6261,7 +6252,7 @@
         <v>160</v>
       </c>
       <c r="E122" s="21" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="F122" s="17"/>
       <c r="G122" s="22"/>
@@ -6296,7 +6287,7 @@
         <v>161</v>
       </c>
       <c r="E123" s="21" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="F123" s="17"/>
       <c r="G123" s="22"/>
@@ -6331,7 +6322,7 @@
         <v>162</v>
       </c>
       <c r="E124" s="21" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="F124" s="17"/>
       <c r="G124" s="22"/>
@@ -6452,7 +6443,7 @@
       </c>
       <c r="E127" s="10"/>
       <c r="F127" s="21" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="G127" s="22">
         <v>4</v>
@@ -6460,15 +6451,15 @@
       <c r="H127" s="10"/>
       <c r="I127" s="12">
         <f t="shared" si="20"/>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="J127" s="12">
         <f t="shared" si="21"/>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="K127" s="12">
         <f t="shared" si="22"/>
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="L127" s="18"/>
       <c r="M127" s="18"/>
@@ -8055,19 +8046,19 @@
       <c r="H170" s="10"/>
       <c r="I170" s="38">
         <f t="shared" ref="I170:K170" si="24">SUM(I4:I162)</f>
-        <v>84</v>
+        <v>96</v>
       </c>
       <c r="J170" s="12">
         <f t="shared" si="24"/>
-        <v>70</v>
+        <v>78</v>
       </c>
       <c r="K170" s="12">
         <f t="shared" si="24"/>
-        <v>67</v>
+        <v>78</v>
       </c>
       <c r="L170" s="12">
         <f>CHOOSE(SUM(L165:L168)+1, MIN(60, K170) + (K170 - MIN(60, K170))/2,MIN(70, KJ170) + (K170 - MIN(70, K170))/2,MIN(80, K170) + (K170 - MIN(80, K170))/2,MIN(90, K170) + (K170 - MIN(90, K170))/2, K170)</f>
-        <v>63.5</v>
+        <v>69</v>
       </c>
       <c r="M170" s="18"/>
       <c r="N170" s="7"/>

</xml_diff>